<commit_message>
T2278 changes 15 july 24
</commit_message>
<xml_diff>
--- a/TestData/LV_T2278_EventExpenseEmailNotificationRequestMoreInformationApproveAsFirstLevelApproverSet2.xlsx
+++ b/TestData/LV_T2278_EventExpenseEmailNotificationRequestMoreInformationApproveAsFirstLevelApproverSet2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E54582-F354-4485-A61C-C21C4622504E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1444BEA-C549-437F-A728-A52843B28BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Users" sheetId="2" r:id="rId1"/>
     <sheet name="AppName" sheetId="4" r:id="rId2"/>
     <sheet name="ModuleName" sheetId="5" r:id="rId3"/>
-    <sheet name="ExpenseRequest" sheetId="1" r:id="rId4"/>
+    <sheet name="EventExp" sheetId="1" r:id="rId4"/>
     <sheet name="Approver" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>

</xml_diff>